<commit_message>
docs: add production planning GSA tutorial with Sobol example
</commit_message>
<xml_diff>
--- a/docs/source/tutorials/production_planning_gsa/materials/model/results/GSA_analysis.xlsx
+++ b/docs/source/tutorials/production_planning_gsa/materials/model/results/GSA_analysis.xlsx
@@ -463,7 +463,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -483,7 +483,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -493,7 +493,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -513,17 +513,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>23.47783251231525</v>
+        <v>0.4353583233422971</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -553,7 +553,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -573,17 +573,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>24.21182266009851</v>
+        <v>0.4649841353724661</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -613,7 +613,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -633,17 +633,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>23.47783251231525</v>
+        <v>0.1800592272591068</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -673,7 +673,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -693,17 +693,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>24.21182266009851</v>
+        <v>0.1394531873801475</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -733,7 +733,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -753,17 +753,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>19.02724123702999</v>
+        <v>0.5232588771135137</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -793,7 +793,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -813,17 +813,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>18.31410304211904</v>
+        <v>0.5394054043564355</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -853,7 +853,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -873,17 +873,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>11.42675687891568</v>
+        <v>0.189590338400917</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -903,7 +903,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -913,7 +913,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -933,17 +933,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>9.735005406759877</v>
+        <v>0.1542172352711496</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -973,7 +973,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1003,7 +1003,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1023,17 +1023,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>39.99999999999999</v>
+        <v>0.9825556387426618</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F21" t="n">
@@ -1063,7 +1063,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1083,7 +1083,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1093,7 +1093,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1123,7 +1123,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1143,17 +1143,17 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>39.99999999999999</v>
+        <v>0.2280898685637951</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1183,7 +1183,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F26" t="n">
@@ -1213,7 +1213,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F27" t="n">
@@ -1243,7 +1243,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1263,17 +1263,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>7.489778066296963e-15</v>
+        <v>0.9868159273354572</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1293,7 +1293,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -1303,7 +1303,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F30" t="n">
@@ -1333,7 +1333,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -1363,7 +1363,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1383,17 +1383,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1.399654025397635e-14</v>
+        <v>0.189980931311943</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -1423,7 +1423,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1443,17 +1443,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>62.85714285714287</v>
+        <v>0.9622642656734991</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -1483,7 +1483,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1503,7 +1503,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -1513,7 +1513,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -1543,7 +1543,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1563,17 +1563,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>62.85714285714287</v>
+        <v>0.1940591782468827</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -1603,7 +1603,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -1633,7 +1633,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -1663,7 +1663,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1683,17 +1683,17 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>2.721171505744275e-14</v>
+        <v>0.9652871843862046</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1713,7 +1713,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -1723,7 +1723,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -1753,7 +1753,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1773,7 +1773,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -1783,7 +1783,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1803,17 +1803,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4.080657645760096e-14</v>
+        <v>0.1798997053094837</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -1843,7 +1843,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1863,7 +1863,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -1873,7 +1873,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1893,7 +1893,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F49" t="n">
@@ -1903,7 +1903,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1923,17 +1923,17 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>58.33990147783253</v>
+        <v>0.9213527714298642</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -1963,7 +1963,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1983,17 +1983,17 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>8.374384236453206</v>
+        <v>0.0110227865983682</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2013,7 +2013,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>mu</t>
+          <t>S1</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -2023,7 +2023,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2043,17 +2043,17 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>58.33990147783253</v>
+        <v>0.1905866084858567</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2073,7 +2073,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -2083,7 +2083,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2103,17 +2103,17 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>8.374384236453206</v>
+        <v>0.04666271185495452</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>mu_star</t>
+          <t>S1_conf</t>
         </is>
       </c>
       <c r="F57" t="n">
@@ -2143,7 +2143,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2163,17 +2163,17 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>6.46970776701693</v>
+        <v>0.9514527212331638</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F59" t="n">
@@ -2203,7 +2203,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2223,17 +2223,17 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F60" t="n">
-        <v>9.172796515343427</v>
+        <v>0.03362215107326826</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>sigma</t>
+          <t>ST</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -2263,7 +2263,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2283,17 +2283,17 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F62" t="n">
-        <v>3.459799053385314</v>
+        <v>0.1773508744935151</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2313,7 +2313,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -2323,7 +2323,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2343,17 +2343,17 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F64" t="n">
-        <v>5.933964933570508</v>
+        <v>0.01990597369935455</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>morris</t>
+          <t>sobol</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>mu_star_conf</t>
+          <t>ST_conf</t>
         </is>
       </c>
       <c r="F65" t="n">

</xml_diff>